<commit_message>
Add Reebelo direct matching & color aliasing
Introduce a deterministic direct-match fast path for nested stores (Reebelo) to avoid AI false-negatives: add matchDirectly in ReebeloSearchService and wire it into processSingleProduct to bypass Gemini when available. Improve Reebelo variant handling: enforce correct selection order (storage → color → condition → battery → SIM), add clickReebeloVariant with multiple selection strategies and color alias expansion, and make variant selection more robust with clearer error handling. Enhance Gemini matcher: introduce a color alias map and update prompt/rules to allow brand-prefixed color equivalence, add MAX_CANDIDATES logic for candidate selection, and strengthen color-check logic. Misc: adjust DOM inspection flow and update output/input sample files to reflect a matched Reebelo result.
</commit_message>
<xml_diff>
--- a/output/reebelo_2026-06-12.xlsx
+++ b/output/reebelo_2026-06-12.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,123 +430,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SGlxZFld5512GBIBlu-VR-ASN-AU</v>
+        <v>SM25UT512GBGry-RD-VR-EXD-AU</v>
       </c>
       <c r="B2" t="str">
-        <v>Samsung Galaxy Z Fold 5 (512GB, Icy Blue) - Pristine</v>
+        <v>Samsung Galaxy S25 Ultra 5G (512GB, Gray) - Excellent</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>https://reebelo.com.au/collections/galaxy-s25-ultra?skuId=sku-mip9jiqdsIKY0wapXN4Ngfv</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>https://reebelo.com.au/collections/galaxy-s25-ultra?skuId=sku-mip9jiqdsIKY0wapXN4Ngfv</v>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>Galaxy S25 Ultra - 512GB - Titanium Gray</v>
       </c>
       <c r="G2" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="str">
-        <v>no_match</v>
+        <v>matched</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>SGlxZFld5512GBIBluAS-VR-ASN-AU</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Samsung Galaxy Z Fold 5 (512GB, Icy Blue) Australian Stock - Pristine</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v>0</v>
-      </c>
-      <c r="H3" t="str">
-        <v>no_match</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>SGlxZFld51TBBlk-VR-ASN-AU</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Samsung Galaxy Z Fold 5 5G (1TB, Black) - Pristine</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>0</v>
-      </c>
-      <c r="H4" t="str">
-        <v>no_match</v>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>SGlxZFld51TBBlkAS-VR-ASN-AU</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Samsung Galaxy Z Fold 5 5G (1TB, Black) Australian Stock - Pristine</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v>0</v>
-      </c>
-      <c r="H5" t="str">
-        <v>no_match</v>
-      </c>
-      <c r="I5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>